<commit_message>
inicia financieras no bancos
</commit_message>
<xml_diff>
--- a/Valuaciones_USA/CI_score_ponderados.xlsx
+++ b/Valuaciones_USA/CI_score_ponderados.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>% importancia</t>
   </si>
@@ -79,9 +79,18 @@
     <t>Sep2025</t>
   </si>
   <si>
+    <t>Amortizacion(%)</t>
+  </si>
+  <si>
     <t>Net Profit Margin(%)</t>
   </si>
   <si>
+    <t>Gross Profit(%)</t>
+  </si>
+  <si>
+    <t>Operating Margin(%)</t>
+  </si>
+  <si>
     <t>EPS</t>
   </si>
   <si>
@@ -91,7 +100,7 @@
     <t># Shares</t>
   </si>
   <si>
-    <t>Net Interest Margin (Bank Only) %</t>
+    <t>Inventory Turnover Ratio</t>
   </si>
   <si>
     <t>Dividends per Share</t>
@@ -112,12 +121,21 @@
     <t>Pasivo/Fondos Propios</t>
   </si>
   <si>
+    <t>Current Ratio</t>
+  </si>
+  <si>
     <t>long-term debt-to-equity(%)</t>
   </si>
   <si>
     <t>Gasto financiero(%)</t>
   </si>
   <si>
+    <t>Inventory to current Assets(%)</t>
+  </si>
+  <si>
+    <t>Net Trading Cycle</t>
+  </si>
+  <si>
     <t>PEGY Ratio</t>
   </si>
   <si>
@@ -127,6 +145,9 @@
     <t>P/S Ratio</t>
   </si>
   <si>
+    <t>Receivable to Current Assets(%)</t>
+  </si>
+  <si>
     <t>ROA%</t>
   </si>
   <si>
@@ -136,28 +157,22 @@
     <t>ROB</t>
   </si>
   <si>
+    <t>ROIC %</t>
+  </si>
+  <si>
     <t>WACC %</t>
   </si>
   <si>
-    <t>WACC % Growth</t>
+    <t>Test de Acidez</t>
   </si>
   <si>
     <t>Piotrivski F-Score</t>
   </si>
   <si>
+    <t>Altman Z score</t>
+  </si>
+  <si>
     <t>Beneish M-Score</t>
-  </si>
-  <si>
-    <t>Return-on-Tangible-Equity</t>
-  </si>
-  <si>
-    <t>Efficiency Ratio(%)</t>
-  </si>
-  <si>
-    <t>Equity-to-Asset</t>
-  </si>
-  <si>
-    <t>Loan to Deposit Ratio(%)</t>
   </si>
   <si>
     <t>Score Total</t>
@@ -518,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -591,67 +606,7 @@
         <v>21</v>
       </c>
       <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>1</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -659,64 +614,67 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>1.25</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="O3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="P3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="R3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="S3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="T3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="U3">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="V3">
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -724,64 +682,7 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-      <c r="N4">
-        <v>1</v>
-      </c>
-      <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="P4">
-        <v>1</v>
-      </c>
-      <c r="Q4">
-        <v>1</v>
-      </c>
-      <c r="R4">
-        <v>1</v>
-      </c>
-      <c r="S4">
-        <v>1</v>
-      </c>
-      <c r="T4">
-        <v>1</v>
-      </c>
-      <c r="U4">
-        <v>1</v>
-      </c>
-      <c r="V4">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -789,64 +690,7 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>0.5</v>
-      </c>
-      <c r="I5">
-        <v>0.5</v>
-      </c>
-      <c r="J5">
-        <v>0.5</v>
-      </c>
-      <c r="K5">
-        <v>0.5</v>
-      </c>
-      <c r="L5">
-        <v>0.5</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>1</v>
-      </c>
-      <c r="O5">
-        <v>0.5</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>1</v>
-      </c>
-      <c r="U5">
-        <v>1</v>
-      </c>
-      <c r="V5">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -856,70 +700,127 @@
       <c r="B6">
         <v>4</v>
       </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="N6">
+        <v>4</v>
+      </c>
+      <c r="O6">
+        <v>4</v>
+      </c>
+      <c r="P6">
+        <v>4</v>
+      </c>
+      <c r="Q6">
+        <v>4</v>
+      </c>
+      <c r="R6">
+        <v>4</v>
+      </c>
+      <c r="S6">
+        <v>4</v>
+      </c>
+      <c r="T6">
+        <v>4</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:22">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="L7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="M7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="N7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="O7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="P7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="Q7">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="R7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -927,52 +828,49 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>4</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="L8">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="O8">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="P8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <v>0</v>
@@ -981,13 +879,13 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="U8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="V8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -995,22 +893,22 @@
         <v>28</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1025,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="M9">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="N9">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="O9">
         <v>0</v>
@@ -1063,67 +961,64 @@
         <v>29</v>
       </c>
       <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -1131,28 +1026,25 @@
         <v>30</v>
       </c>
       <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="D11">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F11">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -1161,16 +1053,16 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -1202,64 +1094,64 @@
         <v>5</v>
       </c>
       <c r="C12">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L12">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="M12">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="N12">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="O12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V12">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -1267,67 +1159,67 @@
         <v>32</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V13">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -1337,16 +1229,133 @@
       <c r="B14">
         <v>3</v>
       </c>
+      <c r="C14">
+        <v>0.75</v>
+      </c>
+      <c r="D14">
+        <v>0.75</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0.75</v>
+      </c>
+      <c r="G14">
+        <v>0.75</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
       </c>
       <c r="T15">
-        <v>0.5</v>
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -1354,67 +1363,7 @@
         <v>35</v>
       </c>
       <c r="B16">
-        <v>3</v>
-      </c>
-      <c r="C16">
-        <v>2.25</v>
-      </c>
-      <c r="D16">
-        <v>2.25</v>
-      </c>
-      <c r="E16">
-        <v>2.25</v>
-      </c>
-      <c r="F16">
-        <v>3</v>
-      </c>
-      <c r="G16">
-        <v>3</v>
-      </c>
-      <c r="H16">
-        <v>2.25</v>
-      </c>
-      <c r="I16">
-        <v>2.25</v>
-      </c>
-      <c r="J16">
-        <v>2.25</v>
-      </c>
-      <c r="K16">
-        <v>2.25</v>
-      </c>
-      <c r="L16">
-        <v>2.25</v>
-      </c>
-      <c r="M16">
-        <v>2.25</v>
-      </c>
-      <c r="N16">
-        <v>2.25</v>
-      </c>
-      <c r="O16">
-        <v>2.25</v>
-      </c>
-      <c r="P16">
-        <v>2.25</v>
-      </c>
-      <c r="Q16">
-        <v>2.25</v>
-      </c>
-      <c r="R16">
-        <v>2.25</v>
-      </c>
-      <c r="S16">
-        <v>2.25</v>
-      </c>
-      <c r="T16">
-        <v>2.25</v>
-      </c>
-      <c r="U16">
-        <v>2.25</v>
-      </c>
-      <c r="V16">
-        <v>2.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:22">
@@ -1422,28 +1371,28 @@
         <v>36</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -1452,37 +1401,37 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="M17">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="N17">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="O17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V17">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -1490,67 +1439,7 @@
         <v>37</v>
       </c>
       <c r="B18">
-        <v>6</v>
-      </c>
-      <c r="C18">
-        <v>6</v>
-      </c>
-      <c r="D18">
-        <v>6</v>
-      </c>
-      <c r="E18">
-        <v>1.5</v>
-      </c>
-      <c r="F18">
-        <v>6</v>
-      </c>
-      <c r="G18">
-        <v>6</v>
-      </c>
-      <c r="H18">
-        <v>6</v>
-      </c>
-      <c r="I18">
-        <v>6</v>
-      </c>
-      <c r="J18">
-        <v>6</v>
-      </c>
-      <c r="K18">
-        <v>6</v>
-      </c>
-      <c r="L18">
-        <v>6</v>
-      </c>
-      <c r="M18">
-        <v>6</v>
-      </c>
-      <c r="N18">
-        <v>6</v>
-      </c>
-      <c r="O18">
-        <v>6</v>
-      </c>
-      <c r="P18">
-        <v>6</v>
-      </c>
-      <c r="Q18">
-        <v>6</v>
-      </c>
-      <c r="R18">
-        <v>6</v>
-      </c>
-      <c r="S18">
-        <v>6</v>
-      </c>
-      <c r="T18">
-        <v>6</v>
-      </c>
-      <c r="U18">
-        <v>6</v>
-      </c>
-      <c r="V18">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -1558,67 +1447,7 @@
         <v>38</v>
       </c>
       <c r="B19">
-        <v>8</v>
-      </c>
-      <c r="C19">
-        <v>8</v>
-      </c>
-      <c r="D19">
-        <v>8</v>
-      </c>
-      <c r="E19">
-        <v>2</v>
-      </c>
-      <c r="F19">
-        <v>8</v>
-      </c>
-      <c r="G19">
-        <v>8</v>
-      </c>
-      <c r="H19">
-        <v>6</v>
-      </c>
-      <c r="I19">
-        <v>6</v>
-      </c>
-      <c r="J19">
-        <v>6</v>
-      </c>
-      <c r="K19">
-        <v>6</v>
-      </c>
-      <c r="L19">
-        <v>6</v>
-      </c>
-      <c r="M19">
-        <v>6</v>
-      </c>
-      <c r="N19">
-        <v>6</v>
-      </c>
-      <c r="O19">
-        <v>2</v>
-      </c>
-      <c r="P19">
-        <v>2</v>
-      </c>
-      <c r="Q19">
-        <v>6</v>
-      </c>
-      <c r="R19">
-        <v>2</v>
-      </c>
-      <c r="S19">
-        <v>6</v>
-      </c>
-      <c r="T19">
-        <v>2</v>
-      </c>
-      <c r="U19">
-        <v>2</v>
-      </c>
-      <c r="V19">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -1626,67 +1455,7 @@
         <v>39</v>
       </c>
       <c r="B20">
-        <v>2</v>
-      </c>
-      <c r="C20">
-        <v>2</v>
-      </c>
-      <c r="D20">
-        <v>2</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>2</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20">
-        <v>2</v>
-      </c>
-      <c r="I20">
-        <v>2</v>
-      </c>
-      <c r="J20">
-        <v>2</v>
-      </c>
-      <c r="K20">
-        <v>2</v>
-      </c>
-      <c r="L20">
-        <v>2</v>
-      </c>
-      <c r="M20">
-        <v>2</v>
-      </c>
-      <c r="N20">
-        <v>2</v>
-      </c>
-      <c r="O20">
-        <v>2</v>
-      </c>
-      <c r="P20">
-        <v>2</v>
-      </c>
-      <c r="Q20">
-        <v>2</v>
-      </c>
-      <c r="R20">
-        <v>2</v>
-      </c>
-      <c r="S20">
-        <v>2</v>
-      </c>
-      <c r="T20">
-        <v>2</v>
-      </c>
-      <c r="U20">
-        <v>2</v>
-      </c>
-      <c r="V20">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -1694,67 +1463,10 @@
         <v>40</v>
       </c>
       <c r="B21">
-        <v>2</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21">
-        <v>1</v>
-      </c>
-      <c r="H21">
-        <v>2</v>
-      </c>
-      <c r="I21">
-        <v>2</v>
-      </c>
-      <c r="J21">
-        <v>2</v>
-      </c>
-      <c r="K21">
-        <v>2</v>
-      </c>
-      <c r="L21">
-        <v>2</v>
-      </c>
-      <c r="M21">
-        <v>2</v>
-      </c>
-      <c r="N21">
-        <v>2</v>
-      </c>
-      <c r="O21">
-        <v>1</v>
-      </c>
-      <c r="P21">
-        <v>2</v>
-      </c>
-      <c r="Q21">
-        <v>2</v>
-      </c>
-      <c r="R21">
-        <v>2</v>
-      </c>
-      <c r="S21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21">
-        <v>2</v>
-      </c>
-      <c r="U21">
-        <v>2</v>
-      </c>
-      <c r="V21">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -1762,67 +1474,67 @@
         <v>41</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="F22">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="J22">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="M22">
-        <v>0.5</v>
+        <v>3.75</v>
       </c>
       <c r="N22">
-        <v>0.5</v>
+        <v>3.75</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="P22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="Q22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="R22">
-        <v>0.5</v>
+        <v>3.75</v>
       </c>
       <c r="S22">
-        <v>0.5</v>
+        <v>3.75</v>
       </c>
       <c r="T22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="U22">
-        <v>0.5</v>
+        <v>3.75</v>
       </c>
       <c r="V22">
-        <v>1</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="23" spans="1:22">
@@ -1830,67 +1542,67 @@
         <v>42</v>
       </c>
       <c r="B23">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C23">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="D23">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="F23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="H23">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="K23">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L23">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M23">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N23">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O23">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="P23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="Q23">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="S23">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="T23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="U23">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="V23">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:22">
@@ -1898,67 +1610,7 @@
         <v>43</v>
       </c>
       <c r="B24">
-        <v>5</v>
-      </c>
-      <c r="C24">
-        <v>5</v>
-      </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-      <c r="E24">
-        <v>5</v>
-      </c>
-      <c r="F24">
-        <v>5</v>
-      </c>
-      <c r="G24">
-        <v>5</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
-      <c r="I24">
-        <v>5</v>
-      </c>
-      <c r="J24">
-        <v>5</v>
-      </c>
-      <c r="K24">
-        <v>5</v>
-      </c>
-      <c r="L24">
-        <v>5</v>
-      </c>
-      <c r="M24">
-        <v>5</v>
-      </c>
-      <c r="N24">
-        <v>5</v>
-      </c>
-      <c r="O24">
-        <v>5</v>
-      </c>
-      <c r="P24">
-        <v>5</v>
-      </c>
-      <c r="Q24">
-        <v>5</v>
-      </c>
-      <c r="R24">
-        <v>5</v>
-      </c>
-      <c r="S24">
-        <v>5</v>
-      </c>
-      <c r="T24">
-        <v>5</v>
-      </c>
-      <c r="U24">
-        <v>5</v>
-      </c>
-      <c r="V24">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:22">
@@ -1966,43 +1618,67 @@
         <v>44</v>
       </c>
       <c r="B25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N25">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="O25">
+        <v>1</v>
+      </c>
+      <c r="P25">
+        <v>1</v>
+      </c>
+      <c r="Q25">
+        <v>1</v>
+      </c>
+      <c r="R25">
+        <v>1</v>
+      </c>
+      <c r="S25">
+        <v>1</v>
+      </c>
+      <c r="T25">
+        <v>1</v>
+      </c>
+      <c r="U25">
+        <v>1</v>
+      </c>
+      <c r="V25">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -2010,7 +1686,67 @@
         <v>45</v>
       </c>
       <c r="B26">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>6</v>
+      </c>
+      <c r="E26">
+        <v>1.5</v>
+      </c>
+      <c r="F26">
+        <v>6</v>
+      </c>
+      <c r="G26">
+        <v>6</v>
+      </c>
+      <c r="H26">
+        <v>4.5</v>
+      </c>
+      <c r="I26">
+        <v>4.5</v>
+      </c>
+      <c r="J26">
+        <v>1.5</v>
+      </c>
+      <c r="K26">
+        <v>4.5</v>
+      </c>
+      <c r="L26">
+        <v>4.5</v>
+      </c>
+      <c r="M26">
+        <v>1.5</v>
+      </c>
+      <c r="N26">
+        <v>4.5</v>
+      </c>
+      <c r="O26">
+        <v>1.5</v>
+      </c>
+      <c r="P26">
+        <v>1.5</v>
+      </c>
+      <c r="Q26">
+        <v>4.5</v>
+      </c>
+      <c r="R26">
+        <v>1.5</v>
+      </c>
+      <c r="S26">
+        <v>1.5</v>
+      </c>
+      <c r="T26">
+        <v>1.5</v>
+      </c>
+      <c r="U26">
+        <v>1.5</v>
+      </c>
+      <c r="V26">
+        <v>1.5</v>
       </c>
     </row>
     <row r="27" spans="1:22">
@@ -2018,67 +1754,67 @@
         <v>46</v>
       </c>
       <c r="B27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="C27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="N27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="O27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="P27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="Q27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="R27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="S27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="T27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="U27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="V27">
-        <v>7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="28" spans="1:22">
@@ -2086,7 +1822,67 @@
         <v>47</v>
       </c>
       <c r="B28">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
+        <v>5</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28">
+        <v>5</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>5</v>
+      </c>
+      <c r="T28">
+        <v>5</v>
+      </c>
+      <c r="U28">
+        <v>0</v>
+      </c>
+      <c r="V28">
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:22">
@@ -2094,67 +1890,227 @@
         <v>48</v>
       </c>
       <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22">
+      <c r="A30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
+      <c r="A31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31">
+        <v>5</v>
+      </c>
+      <c r="C31">
+        <v>2.5</v>
+      </c>
+      <c r="D31">
+        <v>5</v>
+      </c>
+      <c r="E31">
+        <v>2.5</v>
+      </c>
+      <c r="F31">
+        <v>2.5</v>
+      </c>
+      <c r="G31">
+        <v>2.5</v>
+      </c>
+      <c r="H31">
+        <v>2.5</v>
+      </c>
+      <c r="I31">
+        <v>5</v>
+      </c>
+      <c r="J31">
+        <v>2.5</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+      <c r="L31">
+        <v>5</v>
+      </c>
+      <c r="M31">
+        <v>5</v>
+      </c>
+      <c r="N31">
+        <v>5</v>
+      </c>
+      <c r="O31">
+        <v>5</v>
+      </c>
+      <c r="P31">
+        <v>2.5</v>
+      </c>
+      <c r="Q31">
+        <v>5</v>
+      </c>
+      <c r="R31">
+        <v>2.5</v>
+      </c>
+      <c r="S31">
+        <v>5</v>
+      </c>
+      <c r="T31">
+        <v>2.5</v>
+      </c>
+      <c r="U31">
+        <v>2.5</v>
+      </c>
+      <c r="V31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
+      <c r="A32" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22">
+      <c r="A33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>1</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
+        <v>1</v>
+      </c>
+      <c r="M33">
+        <v>1</v>
+      </c>
+      <c r="N33">
+        <v>1</v>
+      </c>
+      <c r="O33">
+        <v>1</v>
+      </c>
+      <c r="P33">
+        <v>1</v>
+      </c>
+      <c r="Q33">
+        <v>1</v>
+      </c>
+      <c r="R33">
+        <v>1</v>
+      </c>
+      <c r="S33">
+        <v>1</v>
+      </c>
+      <c r="T33">
+        <v>1</v>
+      </c>
+      <c r="U33">
+        <v>1</v>
+      </c>
+      <c r="V33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22">
+      <c r="A34" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34">
         <v>100</v>
       </c>
-      <c r="C29">
-        <v>50.75</v>
-      </c>
-      <c r="D29">
-        <v>62.5</v>
-      </c>
-      <c r="E29">
-        <v>35.05</v>
-      </c>
-      <c r="F29">
-        <v>57.5</v>
-      </c>
-      <c r="G29">
-        <v>60.3</v>
-      </c>
-      <c r="H29">
-        <v>49.75</v>
-      </c>
-      <c r="I29">
-        <v>59.25</v>
-      </c>
-      <c r="J29">
-        <v>51.75</v>
-      </c>
-      <c r="K29">
-        <v>57.25</v>
-      </c>
-      <c r="L29">
-        <v>58.55</v>
-      </c>
-      <c r="M29">
-        <v>59</v>
-      </c>
-      <c r="N29">
-        <v>59</v>
-      </c>
-      <c r="O29">
-        <v>47.25</v>
-      </c>
-      <c r="P29">
-        <v>45.25</v>
-      </c>
-      <c r="Q29">
-        <v>53.75</v>
-      </c>
-      <c r="R29">
-        <v>46.25</v>
-      </c>
-      <c r="S29">
-        <v>53.75</v>
-      </c>
-      <c r="T29">
-        <v>49.25</v>
-      </c>
-      <c r="U29">
-        <v>44.25</v>
-      </c>
-      <c r="V29">
-        <v>55.25</v>
+      <c r="C34">
+        <v>19.75</v>
+      </c>
+      <c r="D34">
+        <v>39</v>
+      </c>
+      <c r="E34">
+        <v>25</v>
+      </c>
+      <c r="F34">
+        <v>33.5</v>
+      </c>
+      <c r="G34">
+        <v>38</v>
+      </c>
+      <c r="H34">
+        <v>20.75</v>
+      </c>
+      <c r="I34">
+        <v>32.25</v>
+      </c>
+      <c r="J34">
+        <v>17.75</v>
+      </c>
+      <c r="K34">
+        <v>23.25</v>
+      </c>
+      <c r="L34">
+        <v>34.25</v>
+      </c>
+      <c r="M34">
+        <v>34.75</v>
+      </c>
+      <c r="N34">
+        <v>41.75</v>
+      </c>
+      <c r="O34">
+        <v>30.75</v>
+      </c>
+      <c r="P34">
+        <v>21</v>
+      </c>
+      <c r="Q34">
+        <v>31.5</v>
+      </c>
+      <c r="R34">
+        <v>22.5</v>
+      </c>
+      <c r="S34">
+        <v>30</v>
+      </c>
+      <c r="T34">
+        <v>29.5</v>
+      </c>
+      <c r="U34">
+        <v>18</v>
+      </c>
+      <c r="V34">
+        <v>30.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se agregan razons para financiers no bancos
</commit_message>
<xml_diff>
--- a/Valuaciones_USA/CI_score_ponderados.xlsx
+++ b/Valuaciones_USA/CI_score_ponderados.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>% importancia</t>
   </si>
@@ -79,18 +79,9 @@
     <t>Sep2025</t>
   </si>
   <si>
-    <t>Amortizacion(%)</t>
-  </si>
-  <si>
     <t>Net Profit Margin(%)</t>
   </si>
   <si>
-    <t>Gross Profit(%)</t>
-  </si>
-  <si>
-    <t>Operating Margin(%)</t>
-  </si>
-  <si>
     <t>EPS</t>
   </si>
   <si>
@@ -100,9 +91,6 @@
     <t># Shares</t>
   </si>
   <si>
-    <t>Inventory Turnover Ratio</t>
-  </si>
-  <si>
     <t>Dividends per Share</t>
   </si>
   <si>
@@ -121,21 +109,9 @@
     <t>Pasivo/Fondos Propios</t>
   </si>
   <si>
-    <t>Current Ratio</t>
-  </si>
-  <si>
     <t>long-term debt-to-equity(%)</t>
   </si>
   <si>
-    <t>Gasto financiero(%)</t>
-  </si>
-  <si>
-    <t>Inventory to current Assets(%)</t>
-  </si>
-  <si>
-    <t>Net Trading Cycle</t>
-  </si>
-  <si>
     <t>PEGY Ratio</t>
   </si>
   <si>
@@ -145,9 +121,6 @@
     <t>P/S Ratio</t>
   </si>
   <si>
-    <t>Receivable to Current Assets(%)</t>
-  </si>
-  <si>
     <t>ROA%</t>
   </si>
   <si>
@@ -163,9 +136,6 @@
     <t>WACC %</t>
   </si>
   <si>
-    <t>Test de Acidez</t>
-  </si>
-  <si>
     <t>Piotrivski F-Score</t>
   </si>
   <si>
@@ -173,6 +143,12 @@
   </si>
   <si>
     <t>Beneish M-Score</t>
+  </si>
+  <si>
+    <t>Loss Ratio(%)</t>
+  </si>
+  <si>
+    <t>Expense Ratio(%)</t>
   </si>
   <si>
     <t>Score Total</t>
@@ -533,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -606,7 +582,67 @@
         <v>21</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>1.25</v>
+      </c>
+      <c r="D2">
+        <v>1.25</v>
+      </c>
+      <c r="E2">
+        <v>1.25</v>
+      </c>
+      <c r="F2">
+        <v>1.25</v>
+      </c>
+      <c r="G2">
+        <v>1.25</v>
+      </c>
+      <c r="H2">
+        <v>1.25</v>
+      </c>
+      <c r="I2">
+        <v>1.25</v>
+      </c>
+      <c r="J2">
+        <v>1.25</v>
+      </c>
+      <c r="K2">
+        <v>1.25</v>
+      </c>
+      <c r="L2">
+        <v>1.25</v>
+      </c>
+      <c r="M2">
+        <v>1.25</v>
+      </c>
+      <c r="N2">
+        <v>1.25</v>
+      </c>
+      <c r="O2">
+        <v>1.25</v>
+      </c>
+      <c r="P2">
+        <v>1.25</v>
+      </c>
+      <c r="Q2">
+        <v>1.25</v>
+      </c>
+      <c r="R2">
+        <v>1.25</v>
+      </c>
+      <c r="S2">
+        <v>1.25</v>
+      </c>
+      <c r="T2">
+        <v>1.25</v>
+      </c>
+      <c r="U2">
+        <v>1.25</v>
+      </c>
+      <c r="V2">
+        <v>1.25</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -614,67 +650,64 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="E3">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="N3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="O3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="P3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="Q3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="R3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="S3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="T3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
       <c r="U3">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="V3">
-        <v>1.25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -682,7 +715,64 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
+      <c r="O4">
+        <v>2</v>
+      </c>
+      <c r="P4">
+        <v>2</v>
+      </c>
+      <c r="Q4">
+        <v>2</v>
+      </c>
+      <c r="R4">
+        <v>2</v>
+      </c>
+      <c r="S4">
+        <v>2</v>
+      </c>
+      <c r="T4">
+        <v>2</v>
+      </c>
+      <c r="U4">
+        <v>2</v>
+      </c>
+      <c r="V4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -690,7 +780,64 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>0.5</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="E5">
+        <v>0.5</v>
+      </c>
+      <c r="F5">
+        <v>0.5</v>
+      </c>
+      <c r="G5">
+        <v>0.5</v>
+      </c>
+      <c r="H5">
+        <v>0.25</v>
+      </c>
+      <c r="I5">
+        <v>0.25</v>
+      </c>
+      <c r="J5">
+        <v>0.25</v>
+      </c>
+      <c r="K5">
+        <v>0.25</v>
+      </c>
+      <c r="L5">
+        <v>0.25</v>
+      </c>
+      <c r="M5">
+        <v>0.5</v>
+      </c>
+      <c r="N5">
+        <v>0.5</v>
+      </c>
+      <c r="O5">
+        <v>0.25</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0.5</v>
+      </c>
+      <c r="U5">
+        <v>0.5</v>
+      </c>
+      <c r="V5">
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -698,64 +845,64 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="N6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="O6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="P6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="Q6">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="R6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -763,64 +910,64 @@
         <v>26</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V7">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -828,43 +975,46 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>0.5</v>
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="E8">
         <v>0.5</v>
       </c>
       <c r="F8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0.5</v>
       </c>
       <c r="H8">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="M8">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="N8">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="O8">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -879,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -893,7 +1043,7 @@
         <v>28</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -941,19 +1091,19 @@
         <v>0</v>
       </c>
       <c r="R9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U9">
         <v>0</v>
       </c>
       <c r="V9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -961,64 +1111,67 @@
         <v>29</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>0.75</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="H10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="P10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -1026,25 +1179,28 @@
         <v>30</v>
       </c>
       <c r="B11">
-        <v>8</v>
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -1053,16 +1209,16 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P11">
         <v>0</v>
@@ -1094,19 +1250,19 @@
         <v>5</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D12">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="E12">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G12">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -1121,13 +1277,13 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="M12">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="N12">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="O12">
         <v>0</v>
@@ -1159,67 +1315,10 @@
         <v>32</v>
       </c>
       <c r="B13">
-        <v>1</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>1</v>
-      </c>
-      <c r="S13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T13">
-        <v>1</v>
-      </c>
-      <c r="U13">
-        <v>0</v>
-      </c>
-      <c r="V13">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -1227,67 +1326,67 @@
         <v>33</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C14">
-        <v>0.75</v>
+        <v>3.75</v>
       </c>
       <c r="D14">
-        <v>0.75</v>
+        <v>3.75</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="F14">
-        <v>0.75</v>
+        <v>5</v>
       </c>
       <c r="G14">
-        <v>0.75</v>
+        <v>5</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="J14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="L14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="M14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="Q14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="S14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="T14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="U14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="V14">
-        <v>0</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -1295,28 +1394,28 @@
         <v>34</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -1328,34 +1427,34 @@
         <v>0</v>
       </c>
       <c r="M15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15">
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -1363,6 +1462,66 @@
         <v>35</v>
       </c>
       <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16">
+        <v>1</v>
+      </c>
+      <c r="T16">
+        <v>1</v>
+      </c>
+      <c r="U16">
+        <v>1</v>
+      </c>
+      <c r="V16">
         <v>1</v>
       </c>
     </row>
@@ -1371,67 +1530,67 @@
         <v>36</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="D17">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F17">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="G17">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="K17">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="L17">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="M17">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="N17">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="U17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="V17">
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -1439,7 +1598,67 @@
         <v>37</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>1.5</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>1.5</v>
+      </c>
+      <c r="N18">
+        <v>1.5</v>
+      </c>
+      <c r="O18">
+        <v>1.5</v>
+      </c>
+      <c r="P18">
+        <v>1.5</v>
+      </c>
+      <c r="Q18">
+        <v>1.5</v>
+      </c>
+      <c r="R18">
+        <v>1.5</v>
+      </c>
+      <c r="S18">
+        <v>1.5</v>
+      </c>
+      <c r="T18">
+        <v>1.5</v>
+      </c>
+      <c r="U18">
+        <v>1.5</v>
+      </c>
+      <c r="V18">
+        <v>1.5</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -1447,7 +1666,67 @@
         <v>38</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>5</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>5</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>5</v>
+      </c>
+      <c r="T19">
+        <v>5</v>
+      </c>
+      <c r="U19">
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -1455,7 +1734,7 @@
         <v>39</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -1463,10 +1742,67 @@
         <v>40</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>2.5</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>2.5</v>
+      </c>
+      <c r="F21">
+        <v>2.5</v>
+      </c>
+      <c r="G21">
+        <v>2.5</v>
+      </c>
+      <c r="H21">
+        <v>2.5</v>
+      </c>
+      <c r="I21">
+        <v>5</v>
+      </c>
+      <c r="J21">
+        <v>2.5</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+      <c r="L21">
+        <v>5</v>
+      </c>
+      <c r="M21">
+        <v>5</v>
+      </c>
+      <c r="N21">
+        <v>5</v>
+      </c>
+      <c r="O21">
+        <v>5</v>
+      </c>
+      <c r="P21">
+        <v>2.5</v>
+      </c>
+      <c r="Q21">
+        <v>5</v>
+      </c>
+      <c r="R21">
+        <v>2.5</v>
+      </c>
+      <c r="S21">
+        <v>5</v>
       </c>
       <c r="T21">
-        <v>1.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="U21">
+        <v>2.5</v>
+      </c>
+      <c r="V21">
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -1476,73 +1812,13 @@
       <c r="B22">
         <v>5</v>
       </c>
-      <c r="C22">
-        <v>3.75</v>
-      </c>
-      <c r="D22">
-        <v>3.75</v>
-      </c>
-      <c r="E22">
-        <v>3.75</v>
-      </c>
-      <c r="F22">
-        <v>5</v>
-      </c>
-      <c r="G22">
-        <v>5</v>
-      </c>
-      <c r="H22">
-        <v>3.75</v>
-      </c>
-      <c r="I22">
-        <v>3.75</v>
-      </c>
-      <c r="J22">
-        <v>3.75</v>
-      </c>
-      <c r="K22">
-        <v>3.75</v>
-      </c>
-      <c r="L22">
-        <v>3.75</v>
-      </c>
-      <c r="M22">
-        <v>3.75</v>
-      </c>
-      <c r="N22">
-        <v>3.75</v>
-      </c>
-      <c r="O22">
-        <v>3.75</v>
-      </c>
-      <c r="P22">
-        <v>3.75</v>
-      </c>
-      <c r="Q22">
-        <v>3.75</v>
-      </c>
-      <c r="R22">
-        <v>3.75</v>
-      </c>
-      <c r="S22">
-        <v>3.75</v>
-      </c>
-      <c r="T22">
-        <v>3.75</v>
-      </c>
-      <c r="U22">
-        <v>3.75</v>
-      </c>
-      <c r="V22">
-        <v>3.75</v>
-      </c>
     </row>
     <row r="23" spans="1:22">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1551,58 +1827,58 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23">
         <v>1</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23">
         <v>1</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23">
         <v>1</v>
       </c>
       <c r="P23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V23">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:22">
@@ -1610,7 +1886,7 @@
         <v>43</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:22">
@@ -1618,67 +1894,7 @@
         <v>44</v>
       </c>
       <c r="B25">
-        <v>4</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25">
-        <v>1</v>
-      </c>
-      <c r="I25">
-        <v>1</v>
-      </c>
-      <c r="J25">
-        <v>1</v>
-      </c>
-      <c r="K25">
-        <v>1</v>
-      </c>
-      <c r="L25">
-        <v>1</v>
-      </c>
-      <c r="M25">
-        <v>1</v>
-      </c>
-      <c r="N25">
-        <v>1</v>
-      </c>
-      <c r="O25">
-        <v>1</v>
-      </c>
-      <c r="P25">
-        <v>1</v>
-      </c>
-      <c r="Q25">
-        <v>1</v>
-      </c>
-      <c r="R25">
-        <v>1</v>
-      </c>
-      <c r="S25">
-        <v>1</v>
-      </c>
-      <c r="T25">
-        <v>1</v>
-      </c>
-      <c r="U25">
-        <v>1</v>
-      </c>
-      <c r="V25">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -1686,430 +1902,66 @@
         <v>45</v>
       </c>
       <c r="B26">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>19.75</v>
       </c>
       <c r="D26">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="E26">
-        <v>1.5</v>
+        <v>25</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>33.5</v>
       </c>
       <c r="G26">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="H26">
-        <v>4.5</v>
+        <v>20.75</v>
       </c>
       <c r="I26">
-        <v>4.5</v>
+        <v>32.25</v>
       </c>
       <c r="J26">
-        <v>1.5</v>
+        <v>17.75</v>
       </c>
       <c r="K26">
-        <v>4.5</v>
+        <v>23.25</v>
       </c>
       <c r="L26">
-        <v>4.5</v>
+        <v>34.25</v>
       </c>
       <c r="M26">
-        <v>1.5</v>
+        <v>34.75</v>
       </c>
       <c r="N26">
-        <v>4.5</v>
+        <v>41.75</v>
       </c>
       <c r="O26">
-        <v>1.5</v>
+        <v>30.75</v>
       </c>
       <c r="P26">
-        <v>1.5</v>
+        <v>21</v>
       </c>
       <c r="Q26">
-        <v>4.5</v>
+        <v>31.5</v>
       </c>
       <c r="R26">
-        <v>1.5</v>
+        <v>22.5</v>
       </c>
       <c r="S26">
-        <v>1.5</v>
+        <v>30</v>
       </c>
       <c r="T26">
-        <v>1.5</v>
+        <v>29.5</v>
       </c>
       <c r="U26">
-        <v>1.5</v>
+        <v>18</v>
       </c>
       <c r="V26">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:22">
-      <c r="A27" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27">
-        <v>1.5</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
-      <c r="M27">
-        <v>1.5</v>
-      </c>
-      <c r="N27">
-        <v>1.5</v>
-      </c>
-      <c r="O27">
-        <v>1.5</v>
-      </c>
-      <c r="P27">
-        <v>1.5</v>
-      </c>
-      <c r="Q27">
-        <v>1.5</v>
-      </c>
-      <c r="R27">
-        <v>1.5</v>
-      </c>
-      <c r="S27">
-        <v>1.5</v>
-      </c>
-      <c r="T27">
-        <v>1.5</v>
-      </c>
-      <c r="U27">
-        <v>1.5</v>
-      </c>
-      <c r="V27">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:22">
-      <c r="A28" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28">
-        <v>10</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
-      <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
-      </c>
-      <c r="I28">
-        <v>0</v>
-      </c>
-      <c r="J28">
-        <v>0</v>
-      </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
-      <c r="L28">
-        <v>0</v>
-      </c>
-      <c r="M28">
-        <v>0</v>
-      </c>
-      <c r="N28">
-        <v>5</v>
-      </c>
-      <c r="O28">
-        <v>0</v>
-      </c>
-      <c r="P28">
-        <v>0</v>
-      </c>
-      <c r="Q28">
-        <v>5</v>
-      </c>
-      <c r="R28">
-        <v>0</v>
-      </c>
-      <c r="S28">
-        <v>5</v>
-      </c>
-      <c r="T28">
-        <v>5</v>
-      </c>
-      <c r="U28">
-        <v>0</v>
-      </c>
-      <c r="V28">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22">
-      <c r="A29" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22">
-      <c r="A30" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22">
-      <c r="A31" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31">
-        <v>5</v>
-      </c>
-      <c r="C31">
-        <v>2.5</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31">
-        <v>2.5</v>
-      </c>
-      <c r="F31">
-        <v>2.5</v>
-      </c>
-      <c r="G31">
-        <v>2.5</v>
-      </c>
-      <c r="H31">
-        <v>2.5</v>
-      </c>
-      <c r="I31">
-        <v>5</v>
-      </c>
-      <c r="J31">
-        <v>2.5</v>
-      </c>
-      <c r="K31">
-        <v>5</v>
-      </c>
-      <c r="L31">
-        <v>5</v>
-      </c>
-      <c r="M31">
-        <v>5</v>
-      </c>
-      <c r="N31">
-        <v>5</v>
-      </c>
-      <c r="O31">
-        <v>5</v>
-      </c>
-      <c r="P31">
-        <v>2.5</v>
-      </c>
-      <c r="Q31">
-        <v>5</v>
-      </c>
-      <c r="R31">
-        <v>2.5</v>
-      </c>
-      <c r="S31">
-        <v>5</v>
-      </c>
-      <c r="T31">
-        <v>2.5</v>
-      </c>
-      <c r="U31">
-        <v>2.5</v>
-      </c>
-      <c r="V31">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:22">
-      <c r="A32" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22">
-      <c r="A33" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33">
-        <v>1</v>
-      </c>
-      <c r="E33">
-        <v>1</v>
-      </c>
-      <c r="F33">
-        <v>1</v>
-      </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-      <c r="H33">
-        <v>0</v>
-      </c>
-      <c r="I33">
-        <v>1</v>
-      </c>
-      <c r="J33">
-        <v>1</v>
-      </c>
-      <c r="K33">
-        <v>1</v>
-      </c>
-      <c r="L33">
-        <v>1</v>
-      </c>
-      <c r="M33">
-        <v>1</v>
-      </c>
-      <c r="N33">
-        <v>1</v>
-      </c>
-      <c r="O33">
-        <v>1</v>
-      </c>
-      <c r="P33">
-        <v>1</v>
-      </c>
-      <c r="Q33">
-        <v>1</v>
-      </c>
-      <c r="R33">
-        <v>1</v>
-      </c>
-      <c r="S33">
-        <v>1</v>
-      </c>
-      <c r="T33">
-        <v>1</v>
-      </c>
-      <c r="U33">
-        <v>1</v>
-      </c>
-      <c r="V33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22">
-      <c r="A34" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B34">
-        <v>100</v>
-      </c>
-      <c r="C34">
-        <v>19.75</v>
-      </c>
-      <c r="D34">
-        <v>39</v>
-      </c>
-      <c r="E34">
-        <v>25</v>
-      </c>
-      <c r="F34">
-        <v>33.5</v>
-      </c>
-      <c r="G34">
-        <v>38</v>
-      </c>
-      <c r="H34">
-        <v>20.75</v>
-      </c>
-      <c r="I34">
-        <v>32.25</v>
-      </c>
-      <c r="J34">
-        <v>17.75</v>
-      </c>
-      <c r="K34">
-        <v>23.25</v>
-      </c>
-      <c r="L34">
-        <v>34.25</v>
-      </c>
-      <c r="M34">
-        <v>34.75</v>
-      </c>
-      <c r="N34">
-        <v>41.75</v>
-      </c>
-      <c r="O34">
-        <v>30.75</v>
-      </c>
-      <c r="P34">
-        <v>21</v>
-      </c>
-      <c r="Q34">
-        <v>31.5</v>
-      </c>
-      <c r="R34">
-        <v>22.5</v>
-      </c>
-      <c r="S34">
-        <v>30</v>
-      </c>
-      <c r="T34">
-        <v>29.5</v>
-      </c>
-      <c r="U34">
-        <v>18</v>
-      </c>
-      <c r="V34">
         <v>30.5</v>
       </c>
     </row>

</xml_diff>